<commit_message>
removed dummy training script
</commit_message>
<xml_diff>
--- a/forecast-video-diffmodels/dataproc/list_of_cyclones.xlsx
+++ b/forecast-video-diffmodels/dataproc/list_of_cyclones.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ren\forecast-diffmodels\dataproc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vedang/Desktop/Rugved Research/forecast-video-diffmodels/dataproc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD02CD5F-7991-412D-91C2-ED1C381434BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A2ABF0-0BD9-A841-8561-06E62F199C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -769,7 +782,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -809,6 +822,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -865,7 +896,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -890,6 +921,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -909,9 +943,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -949,7 +983,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1055,7 +1089,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1197,7 +1231,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1206,19 +1240,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.26953125" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" customWidth="1"/>
-    <col min="3" max="3" width="32.81640625" customWidth="1"/>
-    <col min="4" max="4" width="17.1796875" customWidth="1"/>
-    <col min="5" max="5" width="26.1796875" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="23.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.1640625" customWidth="1"/>
+    <col min="5" max="5" width="26.1640625" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="23.5" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="57" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1244,7 +1278,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1254,7 +1288,7 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="18" t="s">
         <v>11</v>
       </c>
       <c r="E2" t="s">
@@ -1273,7 +1307,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1283,7 +1317,7 @@
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="18" t="s">
         <v>17</v>
       </c>
       <c r="E3" t="s">
@@ -1300,7 +1334,7 @@
       </c>
       <c r="I3" s="10"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1310,7 +1344,7 @@
       <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="18" t="s">
         <v>22</v>
       </c>
       <c r="E4" t="s">
@@ -1329,7 +1363,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1339,7 +1373,7 @@
       <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="18" t="s">
         <v>26</v>
       </c>
       <c r="E5" t="s">
@@ -1356,7 +1390,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1366,7 +1400,7 @@
       <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="18" t="s">
         <v>30</v>
       </c>
       <c r="E6" t="s">
@@ -1385,7 +1419,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1395,7 +1429,7 @@
       <c r="C7" t="s">
         <v>10</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="18" t="s">
         <v>34</v>
       </c>
       <c r="E7" t="s">
@@ -1414,7 +1448,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1424,7 +1458,7 @@
       <c r="C8" t="s">
         <v>10</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="18" t="s">
         <v>37</v>
       </c>
       <c r="E8" t="s">
@@ -1443,11 +1477,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="3"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
@@ -1456,7 +1490,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1466,7 +1500,7 @@
       <c r="C10" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="18" t="s">
         <v>42</v>
       </c>
       <c r="E10" s="11" t="s">
@@ -1485,7 +1519,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1495,7 +1529,7 @@
       <c r="C11" t="s">
         <v>10</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="18" t="s">
         <v>47</v>
       </c>
       <c r="E11" t="s">
@@ -1514,7 +1548,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1524,7 +1558,7 @@
       <c r="C12" t="s">
         <v>10</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="18" t="s">
         <v>52</v>
       </c>
       <c r="E12" t="s">
@@ -1543,7 +1577,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1553,7 +1587,7 @@
       <c r="C13" t="s">
         <v>10</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="18" t="s">
         <v>57</v>
       </c>
       <c r="E13" t="s">
@@ -1570,7 +1604,7 @@
       </c>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1580,7 +1614,7 @@
       <c r="C14" t="s">
         <v>10</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="18" t="s">
         <v>61</v>
       </c>
       <c r="E14" t="s">
@@ -1599,7 +1633,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1609,7 +1643,7 @@
       <c r="C15" t="s">
         <v>10</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="18" t="s">
         <v>65</v>
       </c>
       <c r="E15" t="s">
@@ -1628,7 +1662,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1638,7 +1672,7 @@
       <c r="G16" s="9"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -1648,7 +1682,7 @@
       <c r="C17" t="s">
         <v>71</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="20" t="s">
         <v>72</v>
       </c>
       <c r="E17" t="s">
@@ -1664,7 +1698,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -1674,7 +1708,7 @@
       <c r="C18" t="s">
         <v>71</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="20" t="s">
         <v>76</v>
       </c>
       <c r="E18" t="s">
@@ -1690,7 +1724,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -1700,7 +1734,7 @@
       <c r="C19" t="s">
         <v>71</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="20" t="s">
         <v>81</v>
       </c>
       <c r="E19" t="s">
@@ -1716,7 +1750,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -1726,7 +1760,7 @@
       <c r="C20" t="s">
         <v>71</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="20" t="s">
         <v>85</v>
       </c>
       <c r="E20" t="s">
@@ -1742,7 +1776,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -1752,7 +1786,7 @@
       <c r="C21" t="s">
         <v>71</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="20" t="s">
         <v>89</v>
       </c>
       <c r="E21" t="s">
@@ -1768,7 +1802,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>69</v>
       </c>
@@ -1778,7 +1812,7 @@
       <c r="C22" t="s">
         <v>71</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="20" t="s">
         <v>93</v>
       </c>
       <c r="E22" t="s">
@@ -1794,7 +1828,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1804,7 +1838,7 @@
       <c r="G23" s="9"/>
       <c r="H23" s="4"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>97</v>
       </c>
@@ -1814,7 +1848,7 @@
       <c r="C24" t="s">
         <v>99</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="18" t="s">
         <v>100</v>
       </c>
       <c r="E24" t="s">
@@ -1830,7 +1864,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>97</v>
       </c>
@@ -1840,7 +1874,7 @@
       <c r="C25" t="s">
         <v>99</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="18" t="s">
         <v>104</v>
       </c>
       <c r="E25" t="s">
@@ -1856,7 +1890,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -1866,7 +1900,7 @@
       <c r="C26" t="s">
         <v>99</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="18" t="s">
         <v>108</v>
       </c>
       <c r="E26" t="s">
@@ -1882,7 +1916,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>97</v>
       </c>
@@ -1892,7 +1926,7 @@
       <c r="C27" t="s">
         <v>99</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="18" t="s">
         <v>112</v>
       </c>
       <c r="E27" t="s">
@@ -1908,7 +1942,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>97</v>
       </c>
@@ -1918,7 +1952,7 @@
       <c r="C28" t="s">
         <v>99</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="18" t="s">
         <v>116</v>
       </c>
       <c r="E28" t="s">
@@ -1934,7 +1968,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>97</v>
       </c>
@@ -1944,7 +1978,7 @@
       <c r="C29" t="s">
         <v>99</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="18" t="s">
         <v>120</v>
       </c>
       <c r="E29" t="s">
@@ -1960,7 +1994,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -1970,7 +2004,7 @@
       <c r="C30" t="s">
         <v>99</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="18" t="s">
         <v>124</v>
       </c>
       <c r="E30" t="s">
@@ -1986,7 +2020,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>97</v>
       </c>
@@ -1996,7 +2030,7 @@
       <c r="C31" t="s">
         <v>99</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="18" t="s">
         <v>128</v>
       </c>
       <c r="E31" t="s">
@@ -2012,7 +2046,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2022,7 +2056,7 @@
       <c r="G32" s="9"/>
       <c r="H32" s="4"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>132</v>
       </c>
@@ -2032,7 +2066,7 @@
       <c r="C33" t="s">
         <v>134</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="20" t="s">
         <v>135</v>
       </c>
       <c r="E33" t="s">
@@ -2048,7 +2082,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>132</v>
       </c>
@@ -2058,7 +2092,7 @@
       <c r="C34" t="s">
         <v>134</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="20" t="s">
         <v>139</v>
       </c>
       <c r="E34" t="s">
@@ -2074,7 +2108,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>132</v>
       </c>
@@ -2084,7 +2118,7 @@
       <c r="C35" t="s">
         <v>134</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="20" t="s">
         <v>143</v>
       </c>
       <c r="E35" t="s">
@@ -2100,7 +2134,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>132</v>
       </c>
@@ -2110,7 +2144,7 @@
       <c r="C36" t="s">
         <v>134</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="20" t="s">
         <v>147</v>
       </c>
       <c r="E36" t="s">
@@ -2126,7 +2160,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>132</v>
       </c>
@@ -2136,7 +2170,7 @@
       <c r="C37" t="s">
         <v>134</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="20" t="s">
         <v>151</v>
       </c>
       <c r="E37" t="s">
@@ -2152,7 +2186,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>132</v>
       </c>
@@ -2162,7 +2196,7 @@
       <c r="C38" t="s">
         <v>134</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="20" t="s">
         <v>155</v>
       </c>
       <c r="E38" t="s">
@@ -2178,7 +2212,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>132</v>
       </c>
@@ -2188,7 +2222,7 @@
       <c r="C39" t="s">
         <v>134</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="20" t="s">
         <v>159</v>
       </c>
       <c r="E39" t="s">
@@ -2204,7 +2238,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>132</v>
       </c>
@@ -2214,7 +2248,7 @@
       <c r="C40" t="s">
         <v>134</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="20" t="s">
         <v>163</v>
       </c>
       <c r="E40" t="s">
@@ -2230,7 +2264,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>132</v>
       </c>
@@ -2240,7 +2274,7 @@
       <c r="C41" t="s">
         <v>134</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="20" t="s">
         <v>167</v>
       </c>
       <c r="E41" t="s">
@@ -2256,7 +2290,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>132</v>
       </c>
@@ -2266,7 +2300,7 @@
       <c r="C42" t="s">
         <v>134</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="20" t="s">
         <v>171</v>
       </c>
       <c r="E42" t="s">
@@ -2282,7 +2316,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>132</v>
       </c>
@@ -2292,7 +2326,7 @@
       <c r="C43" t="s">
         <v>134</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="20" t="s">
         <v>175</v>
       </c>
       <c r="E43" t="s">
@@ -2308,7 +2342,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -2318,7 +2352,7 @@
       <c r="G44" s="9"/>
       <c r="H44" s="4"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>179</v>
       </c>
@@ -2328,7 +2362,7 @@
       <c r="C45" t="s">
         <v>181</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="20" t="s">
         <v>182</v>
       </c>
       <c r="E45" t="s">
@@ -2344,7 +2378,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -2354,7 +2388,7 @@
       <c r="C46" t="s">
         <v>181</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="20" t="s">
         <v>186</v>
       </c>
       <c r="E46" t="s">
@@ -2370,7 +2404,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>179</v>
       </c>
@@ -2380,7 +2414,7 @@
       <c r="C47" t="s">
         <v>181</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="20" t="s">
         <v>190</v>
       </c>
       <c r="E47" t="s">
@@ -2396,7 +2430,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>179</v>
       </c>
@@ -2406,7 +2440,7 @@
       <c r="C48" t="s">
         <v>181</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="20" t="s">
         <v>194</v>
       </c>
       <c r="E48" t="s">
@@ -2422,7 +2456,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -2432,7 +2466,7 @@
       <c r="G49" s="9"/>
       <c r="H49" s="4"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>198</v>
       </c>
@@ -2442,7 +2476,7 @@
       <c r="C50" t="s">
         <v>71</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="19" t="s">
         <v>200</v>
       </c>
       <c r="E50" t="s">
@@ -2458,7 +2492,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>198</v>
       </c>
@@ -2468,7 +2502,7 @@
       <c r="C51" t="s">
         <v>71</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="19" t="s">
         <v>203</v>
       </c>
       <c r="E51" t="s">
@@ -2484,7 +2518,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -2494,7 +2528,7 @@
       <c r="C52" t="s">
         <v>71</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" s="20" t="s">
         <v>206</v>
       </c>
       <c r="E52" t="s">
@@ -2510,7 +2544,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>198</v>
       </c>
@@ -2520,7 +2554,7 @@
       <c r="C53" t="s">
         <v>71</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D53" s="19" t="s">
         <v>210</v>
       </c>
       <c r="E53" t="s">
@@ -2536,7 +2570,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>198</v>
       </c>
@@ -2546,7 +2580,7 @@
       <c r="C54" t="s">
         <v>71</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" s="19" t="s">
         <v>214</v>
       </c>
       <c r="E54" t="s">
@@ -2562,7 +2596,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>198</v>
       </c>
@@ -2572,7 +2606,7 @@
       <c r="C55" t="s">
         <v>71</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" s="19" t="s">
         <v>217</v>
       </c>
       <c r="E55" t="s">
@@ -2588,7 +2622,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>198</v>
       </c>
@@ -2598,7 +2632,7 @@
       <c r="C56" t="s">
         <v>71</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="20" t="s">
         <v>221</v>
       </c>
       <c r="E56" t="s">
@@ -2614,7 +2648,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>198</v>
       </c>
@@ -2624,7 +2658,7 @@
       <c r="C57" t="s">
         <v>71</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="19" t="s">
         <v>225</v>
       </c>
       <c r="E57" t="s">
@@ -2640,7 +2674,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>198</v>
       </c>
@@ -2650,7 +2684,7 @@
       <c r="C58" t="s">
         <v>71</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="19" t="s">
         <v>229</v>
       </c>
       <c r="E58" t="s">
@@ -2666,7 +2700,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -2676,13 +2710,13 @@
       <c r="G59" s="9"/>
       <c r="H59" s="4"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E61" s="14" t="s">
         <v>232</v>
       </c>
       <c r="F61"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E62" s="15" t="s">
         <v>233</v>
       </c>
@@ -2691,7 +2725,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E63" s="17" t="s">
         <v>8</v>
       </c>
@@ -2700,7 +2734,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E64" s="17" t="s">
         <v>69</v>
       </c>
@@ -2709,7 +2743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E65" s="17" t="s">
         <v>234</v>
       </c>
@@ -2718,7 +2752,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E66" s="17" t="s">
         <v>132</v>
       </c>
@@ -2727,7 +2761,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E67" s="17" t="s">
         <v>179</v>
       </c>
@@ -2736,7 +2770,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="5:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="5:6" x14ac:dyDescent="0.2">
       <c r="E68" s="17" t="s">
         <v>198</v>
       </c>

</xml_diff>